<commit_message>
Add consumables: stock, expiry, consumption, file upload and requests
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rk5Y94e1axaPVaoX5vmGU
</commit_message>
<xml_diff>
--- a/templates/RTG_data_templates.xlsx
+++ b/templates/RTG_data_templates.xlsx
@@ -6445,7 +6445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6479,6 +6479,131 @@
       <c r="E1" s="4" t="inlineStr">
         <is>
           <t>ReceivedOn</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SAMPLE-A1</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2027-03-31</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-04-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SAMPLE-A2</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SAMPLE-B1</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>14</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2027-06-30</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SAMPLE-D1</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2025-12-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SAMPLE-E1</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>20</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2027-01-31</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FM-led heater return with explanation, readable notification mails, one FM department
FM ticks the parts they hand back, RTG inspects, FM explains damage and the action
they will take, RTG accepts and closes. Notification mails now show the message and
carry the JSON for Power Automate as an attachment.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rk5Y94e1axaPVaoX5vmGU
</commit_message>
<xml_diff>
--- a/templates/RTG_data_templates.xlsx
+++ b/templates/RTG_data_templates.xlsx
@@ -6095,7 +6095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6111,26 +6111,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FM Raw Material</t>
+          <t>FM</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
-        <is>
-          <t>FM Sinter</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>FM Blast Furnace</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
         <is>
           <t>RTG</t>
         </is>

</xml_diff>

<commit_message>
Treat pair heaters as two singles joined, and accept ST ratings
A pair like 14-CD now lists its singles in HeaterModels.MadeFrom and uses
their parts, so it is ready only when both singles are in store, and the
singles show as out while the pair is on site. Find a heater suggests the
guide's ratings for the width, including ST1000/ST1400/ST1600.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rk5Y94e1axaPVaoX5vmGU
</commit_message>
<xml_diff>
--- a/templates/RTG_data_templates.xlsx
+++ b/templates/RTG_data_templates.xlsx
@@ -571,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -584,6 +584,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -637,6 +638,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>MadeFrom</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -675,6 +681,7 @@
           <t>Replace with real data</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -713,6 +720,7 @@
           <t>Replace with real data</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -751,6 +759,7 @@
           <t>Replace with real data</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>